<commit_message>
Updates from the past few days (not previously pushed)
latest data added to raw files, and plot code updated for final version
</commit_message>
<xml_diff>
--- a/RES/tables_revalidation/descriptive_statistics.xlsx
+++ b/RES/tables_revalidation/descriptive_statistics.xlsx
@@ -442,7 +442,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -458,7 +458,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -494,19 +494,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B2" t="n">
-        <v>40.17</v>
+        <v>36.68</v>
       </c>
       <c r="C2" t="n">
-        <v>16.7</v>
+        <v>16.879</v>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -548,13 +548,13 @@
         <v>16</v>
       </c>
       <c r="C2" t="n">
-        <v>85.75</v>
+        <v>81.6315789473684</v>
       </c>
       <c r="D2" t="n">
-        <v>18.61</v>
+        <v>19.55</v>
       </c>
       <c r="E2" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
@@ -565,13 +565,13 @@
         <v>17</v>
       </c>
       <c r="C3" t="n">
-        <v>47.8333333333333</v>
+        <v>48.4210526315789</v>
       </c>
       <c r="D3" t="n">
-        <v>24.59</v>
+        <v>24.12</v>
       </c>
       <c r="E3" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -582,13 +582,13 @@
         <v>18</v>
       </c>
       <c r="C4" t="n">
-        <v>18.0833333333333</v>
+        <v>18.7894736842105</v>
       </c>
       <c r="D4" t="n">
-        <v>21.97</v>
+        <v>19.77</v>
       </c>
       <c r="E4" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -599,13 +599,13 @@
         <v>19</v>
       </c>
       <c r="C5" t="n">
-        <v>14.8333333333333</v>
+        <v>16</v>
       </c>
       <c r="D5" t="n">
-        <v>26.05</v>
+        <v>23.29</v>
       </c>
       <c r="E5" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
@@ -616,13 +616,13 @@
         <v>20</v>
       </c>
       <c r="C6" t="n">
-        <v>21.75</v>
+        <v>29.8421052631579</v>
       </c>
       <c r="D6" t="n">
-        <v>15.36</v>
+        <v>20.42</v>
       </c>
       <c r="E6" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
@@ -633,13 +633,13 @@
         <v>21</v>
       </c>
       <c r="C7" t="n">
-        <v>6.66666666666667</v>
+        <v>7.78947368421053</v>
       </c>
       <c r="D7" t="n">
-        <v>17.2</v>
+        <v>14.7</v>
       </c>
       <c r="E7" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8">
@@ -650,13 +650,13 @@
         <v>16</v>
       </c>
       <c r="C8" t="n">
-        <v>25.9166666666667</v>
+        <v>31</v>
       </c>
       <c r="D8" t="n">
-        <v>23.46</v>
+        <v>27.82</v>
       </c>
       <c r="E8" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
@@ -667,13 +667,13 @@
         <v>17</v>
       </c>
       <c r="C9" t="n">
-        <v>30.0833333333333</v>
+        <v>33.8947368421053</v>
       </c>
       <c r="D9" t="n">
-        <v>30.26</v>
+        <v>26.2</v>
       </c>
       <c r="E9" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">
@@ -684,13 +684,13 @@
         <v>18</v>
       </c>
       <c r="C10" t="n">
-        <v>1.75</v>
+        <v>5.26315789473684</v>
       </c>
       <c r="D10" t="n">
-        <v>1.76</v>
+        <v>15.99</v>
       </c>
       <c r="E10" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
@@ -701,13 +701,13 @@
         <v>19</v>
       </c>
       <c r="C11" t="n">
-        <v>1.5</v>
+        <v>1.42105263157895</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8</v>
+        <v>0.77</v>
       </c>
       <c r="E11" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
@@ -718,13 +718,13 @@
         <v>20</v>
       </c>
       <c r="C12" t="n">
-        <v>69.1666666666667</v>
+        <v>75.1052631578947</v>
       </c>
       <c r="D12" t="n">
-        <v>37.54</v>
+        <v>31.8</v>
       </c>
       <c r="E12" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
@@ -735,13 +735,13 @@
         <v>21</v>
       </c>
       <c r="C13" t="n">
-        <v>73.9166666666667</v>
+        <v>72.8421052631579</v>
       </c>
       <c r="D13" t="n">
-        <v>40.62</v>
+        <v>34.79</v>
       </c>
       <c r="E13" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14">
@@ -752,13 +752,13 @@
         <v>16</v>
       </c>
       <c r="C14" t="n">
-        <v>49.8333333333333</v>
+        <v>57.7894736842105</v>
       </c>
       <c r="D14" t="n">
-        <v>23.3</v>
+        <v>29.12</v>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
@@ -769,13 +769,13 @@
         <v>17</v>
       </c>
       <c r="C15" t="n">
-        <v>60.6666666666667</v>
+        <v>66.7368421052632</v>
       </c>
       <c r="D15" t="n">
-        <v>29.44</v>
+        <v>25.55</v>
       </c>
       <c r="E15" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16">
@@ -786,13 +786,13 @@
         <v>18</v>
       </c>
       <c r="C16" t="n">
-        <v>1.66666666666667</v>
+        <v>2.15789473684211</v>
       </c>
       <c r="D16" t="n">
-        <v>1.78</v>
+        <v>3.2</v>
       </c>
       <c r="E16" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17">
@@ -803,13 +803,13 @@
         <v>19</v>
       </c>
       <c r="C17" t="n">
-        <v>2.83333333333333</v>
+        <v>2.89473684210526</v>
       </c>
       <c r="D17" t="n">
-        <v>4.82</v>
+        <v>4.37</v>
       </c>
       <c r="E17" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18">
@@ -820,13 +820,13 @@
         <v>20</v>
       </c>
       <c r="C18" t="n">
-        <v>67.0833333333333</v>
+        <v>74.2105263157895</v>
       </c>
       <c r="D18" t="n">
-        <v>35.37</v>
+        <v>29.5</v>
       </c>
       <c r="E18" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19">
@@ -837,13 +837,13 @@
         <v>21</v>
       </c>
       <c r="C19" t="n">
-        <v>34.25</v>
+        <v>34.1052631578947</v>
       </c>
       <c r="D19" t="n">
-        <v>33.92</v>
+        <v>30.73</v>
       </c>
       <c r="E19" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20">
@@ -854,13 +854,13 @@
         <v>16</v>
       </c>
       <c r="C20" t="n">
-        <v>25.5</v>
+        <v>26.4736842105263</v>
       </c>
       <c r="D20" t="n">
-        <v>25.33</v>
+        <v>23.53</v>
       </c>
       <c r="E20" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21">
@@ -871,13 +871,13 @@
         <v>17</v>
       </c>
       <c r="C21" t="n">
-        <v>57.8333333333333</v>
+        <v>56.1578947368421</v>
       </c>
       <c r="D21" t="n">
-        <v>34.63</v>
+        <v>31.78</v>
       </c>
       <c r="E21" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22">
@@ -888,13 +888,13 @@
         <v>18</v>
       </c>
       <c r="C22" t="n">
-        <v>3.08333333333333</v>
+        <v>6.05263157894737</v>
       </c>
       <c r="D22" t="n">
-        <v>5.21</v>
+        <v>8.48</v>
       </c>
       <c r="E22" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23">
@@ -905,13 +905,13 @@
         <v>19</v>
       </c>
       <c r="C23" t="n">
-        <v>10.9166666666667</v>
+        <v>10.1052631578947</v>
       </c>
       <c r="D23" t="n">
-        <v>24.97</v>
+        <v>20.96</v>
       </c>
       <c r="E23" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24">
@@ -922,13 +922,13 @@
         <v>20</v>
       </c>
       <c r="C24" t="n">
-        <v>67.75</v>
+        <v>72.8421052631579</v>
       </c>
       <c r="D24" t="n">
-        <v>31.29</v>
+        <v>24.08</v>
       </c>
       <c r="E24" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25">
@@ -939,13 +939,13 @@
         <v>21</v>
       </c>
       <c r="C25" t="n">
-        <v>25.75</v>
+        <v>38.4736842105263</v>
       </c>
       <c r="D25" t="n">
-        <v>26.13</v>
+        <v>33.08</v>
       </c>
       <c r="E25" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26">

</xml_diff>